<commit_message>
Add WF011, real date injection, ID-accuracy rule, tests, regenerated outputs
</commit_message>
<xml_diff>
--- a/data/workflows.xlsx
+++ b/data/workflows.xlsx
@@ -2,16 +2,15 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
-  <workbookProtection/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Workflows" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test_Questions" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="0" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
@@ -27,7 +26,9 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <name val="Calibri"/>
       <b val="1"/>
+      <sz val="11"/>
     </font>
   </fonts>
   <fills count="2">
@@ -47,23 +48,35 @@
       <diagonal/>
     </border>
     <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
     </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
@@ -426,8 +439,8 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H11"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <dimension ref="A1:H12"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
@@ -888,6 +901,48 @@
       <c r="H11" t="inlineStr">
         <is>
           <t>Performance summary with metrics, problem areas, and improvement recommendations</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>WF011</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Overdue Orders Report</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>User asks which orders are overdue, late, delayed, or past their estimated delivery date</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Orders dataset (Order_ID, Status, Shipment_Status, Estimated_Delivery)</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>Load orders data → Compare Estimated_Delivery with today's date → Keep orders where Estimated_Delivery is before today and Status is not Delivered or Cancelled → Calculate days overdue → Format report</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>Flag an order as overdue only if Estimated_Delivery is before today and Status is not Delivered or Cancelled. Orders with no Estimated_Delivery are not flagged. If none are overdue, say so clearly. Do not invent orders.</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>CSV reader; calculator/aggregator; report formatter</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>List of overdue orders with Order_ID, Customer_Name, Status, Estimated_Delivery, and days overdue, plus a total count</t>
         </is>
       </c>
     </row>
@@ -903,7 +958,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:C11"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">

</xml_diff>

<commit_message>
Add WF011 overdue orders, WF009 fix, input file support, README update
</commit_message>
<xml_diff>
--- a/data/workflows.xlsx
+++ b/data/workflows.xlsx
@@ -957,7 +957,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C11"/>
+  <dimension ref="A1:C12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <sheetData>
     <row r="1">
@@ -1121,7 +1121,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Assign this urgent task to the best available developer.</t>
+          <t>Assign this urgent task to the best available developer: fix the payment API timeout bug in our Python FastAPI service.</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -1144,6 +1144,23 @@
       <c r="C11" t="inlineStr">
         <is>
           <t>Tests aggregation and reporting</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>WF011</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Which orders are overdue?</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Tests date comparison and filtering</t>
         </is>
       </c>
     </row>

</xml_diff>